<commit_message>
feat: complete implementing lab
</commit_message>
<xml_diff>
--- a/submissions/2A202602611_BuiVietAnh/code/results.xlsx
+++ b/submissions/2A202602611_BuiVietAnh/code/results.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N2"/>
+  <dimension ref="A1:N3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -535,6 +535,58 @@
         <v>15.27590001933277</v>
       </c>
       <c r="N2" t="inlineStr">
+        <is>
+          <t>Latency: 1 measurement, FP32, excludes preprocessing</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>B02</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>convnext_tiny</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>convnext_tiny.in12k_ft_in1k</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>27.827049</v>
+      </c>
+      <c r="E3" t="n">
+        <v>4.469676288</v>
+      </c>
+      <c r="F3" t="n">
+        <v>224</v>
+      </c>
+      <c r="G3" t="n">
+        <v>12</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" t="n">
+        <v>12</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0.9708122304355147</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0.9768637532133676</v>
+      </c>
+      <c r="L3" t="n">
+        <v>119.6600668583512</v>
+      </c>
+      <c r="M3" t="n">
+        <v>6.346600013785064</v>
+      </c>
+      <c r="N3" t="inlineStr">
         <is>
           <t>Latency: 1 measurement, FP32, excludes preprocessing</t>
         </is>

</xml_diff>